<commit_message>
updated cell referencing and formulas
</commit_message>
<xml_diff>
--- a/Excel Practice @ Day 03 New.xlsx
+++ b/Excel Practice @ Day 03 New.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Codegnan\Data Analytics\Microsoft Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c8f7342ba908387/Desktop/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D7B37C2-DB3D-432E-A6F9-1913D8281B3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{3D7B37C2-DB3D-432E-A6F9-1913D8281B3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{510F71D3-F9B1-47CC-870D-6BB77960EA66}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Patient_Data" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="230">
   <si>
     <t>Patient_ID</t>
   </si>
@@ -982,6 +982,21 @@
       </rPr>
       <t xml:space="preserve"> then MR, NO Review</t>
     </r>
+  </si>
+  <si>
+    <t>payment Alert</t>
+  </si>
+  <si>
+    <t>Bill Category</t>
+  </si>
+  <si>
+    <t>Age Category</t>
+  </si>
+  <si>
+    <t>bill case</t>
+  </si>
+  <si>
+    <t>payment followup</t>
   </si>
 </sst>
 </file>
@@ -1403,31 +1418,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T66"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <dimension ref="A1:V66"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="10.109375" customWidth="1"/>
-    <col min="2" max="2" width="16.21875" customWidth="1"/>
-    <col min="5" max="5" width="19.77734375" customWidth="1"/>
-    <col min="6" max="6" width="15.88671875" customWidth="1"/>
-    <col min="7" max="7" width="18.33203125" customWidth="1"/>
+    <col min="1" max="1" width="10.08984375" customWidth="1"/>
+    <col min="2" max="2" width="16.1796875" customWidth="1"/>
+    <col min="5" max="5" width="19.81640625" customWidth="1"/>
+    <col min="6" max="6" width="15.90625" customWidth="1"/>
+    <col min="7" max="7" width="18.36328125" customWidth="1"/>
     <col min="8" max="8" width="23" customWidth="1"/>
-    <col min="9" max="9" width="16.6640625" customWidth="1"/>
-    <col min="10" max="10" width="19.5546875" customWidth="1"/>
-    <col min="11" max="11" width="16.88671875" customWidth="1"/>
-    <col min="12" max="12" width="18.44140625" customWidth="1"/>
-    <col min="13" max="13" width="16.44140625" customWidth="1"/>
-    <col min="14" max="14" width="15.44140625" customWidth="1"/>
-    <col min="15" max="15" width="14.77734375" customWidth="1"/>
-    <col min="16" max="16" width="15.88671875" customWidth="1"/>
+    <col min="9" max="9" width="16.6328125" customWidth="1"/>
+    <col min="10" max="10" width="19.54296875" customWidth="1"/>
+    <col min="11" max="11" width="16.90625" customWidth="1"/>
+    <col min="12" max="12" width="18.453125" customWidth="1"/>
+    <col min="13" max="13" width="16.453125" customWidth="1"/>
+    <col min="14" max="14" width="15.453125" customWidth="1"/>
+    <col min="15" max="15" width="14.81640625" customWidth="1"/>
+    <col min="16" max="16" width="15.90625" customWidth="1"/>
     <col min="17" max="17" width="21" customWidth="1"/>
-    <col min="18" max="18" width="17.33203125" customWidth="1"/>
-    <col min="19" max="19" width="17.6640625" customWidth="1"/>
-    <col min="20" max="20" width="18.109375" customWidth="1"/>
+    <col min="18" max="18" width="17.36328125" customWidth="1"/>
+    <col min="19" max="19" width="17.6328125" customWidth="1"/>
+    <col min="20" max="20" width="18.08984375" customWidth="1"/>
     <col min="22" max="22" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20">
+    <row r="1" spans="1:22">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1467,15 +1482,28 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="14"/>
-      <c r="O1" s="14"/>
-      <c r="P1" s="14"/>
-      <c r="Q1" s="14"/>
-      <c r="R1" s="14"/>
-      <c r="S1" s="14"/>
+      <c r="N1" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="O1" s="14" t="s">
+        <v>226</v>
+      </c>
+      <c r="P1" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="Q1" s="14" t="s">
+        <v>228</v>
+      </c>
+      <c r="R1" s="14" t="s">
+        <v>229</v>
+      </c>
+      <c r="S1" s="14" t="str">
+        <f>IF(OR(E2="cardiology",E2="neurology"),"priority dep","normal dep")</f>
+        <v>priority dep</v>
+      </c>
       <c r="T1" s="14"/>
     </row>
-    <row r="2" spans="1:20">
+    <row r="2" spans="1:22">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -1515,16 +1543,44 @@
       <c r="M2">
         <v>3</v>
       </c>
+      <c r="N2" t="str">
+        <f>IF(L2="pending","follow-up","no action")</f>
+        <v>no action</v>
+      </c>
+      <c r="O2" t="str">
+        <f>IF(K2&gt;40000,"high bill","normal bill")</f>
+        <v>normal bill</v>
+      </c>
+      <c r="P2" t="str">
+        <f>IF(C2&gt;=60,"senior-citizen","non-senior")</f>
+        <v>non-senior</v>
+      </c>
+      <c r="Q2" t="str">
+        <f>IF(AND(K2&gt;40000,M2&gt;5),"High billing case","normal case")</f>
+        <v>normal case</v>
+      </c>
+      <c r="R2" t="str">
+        <f>IF(AND(L2="pending",K2&gt;30000),"urgent payment follow-up","no action")</f>
+        <v>no action</v>
+      </c>
       <c r="S2" t="str">
-        <f>IF(NOT(L2="Pending"),"Payment Completed","Payment Pending")</f>
-        <v>Payment Completed</v>
+        <f>IF(OR(E2="cardiology",E2="neurology"),"priority dep","normaldep")</f>
+        <v>priority dep</v>
       </c>
       <c r="T2" t="str">
-        <f>IF(AND(OR(Patient_Data!E2="Cardiology",Patient_Data!E2="Orthopedics"),Patient_Data!K2&gt;30000),"MR","NR")</f>
-        <v>NR</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20">
+        <f>IF(NOT(L2="pending"),"paymentdone","paymentnotdone")</f>
+        <v>paymentdone</v>
+      </c>
+      <c r="U2" t="str">
+        <f>IF(K2&lt;15000,"low",IF(K2&lt;=30000,"medium",IF(K2&lt;=50000,"high","very high")))</f>
+        <v>medium</v>
+      </c>
+      <c r="V2" t="str">
+        <f>IF(AND(OR(E2="cardiology",E2="orthopedics"),K2&gt;30000),"management review","noreview")</f>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -1564,8 +1620,44 @@
       <c r="M3">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:20">
+      <c r="N3" t="str">
+        <f t="shared" ref="N3:N41" si="0">IF(L3="pending","follow-up","no action")</f>
+        <v>no action</v>
+      </c>
+      <c r="O3" t="str">
+        <f t="shared" ref="O3:O41" si="1">IF(K3&gt;40000,"high bill","normal bill")</f>
+        <v>high bill</v>
+      </c>
+      <c r="P3" t="str">
+        <f t="shared" ref="P3:P41" si="2">IF(C3&gt;=60,"senior-citizen","non-senior")</f>
+        <v>non-senior</v>
+      </c>
+      <c r="Q3" t="str">
+        <f t="shared" ref="Q3:Q41" si="3">IF(AND(K3&gt;40000,M3&gt;5),"High billing case","normal case")</f>
+        <v>High billing case</v>
+      </c>
+      <c r="R3" t="str">
+        <f>IF(AND(L3="pending",K3&gt;30000),"urgent paymentfollow-up","no action")</f>
+        <v>no action</v>
+      </c>
+      <c r="S3" t="str">
+        <f t="shared" ref="S3:S41" si="4">IF(OR(E3="cardiology",E3="neurology"),"priority dep","normaldep")</f>
+        <v>normaldep</v>
+      </c>
+      <c r="T3" t="str">
+        <f t="shared" ref="T3:T41" si="5">IF(NOT(L3="pending"),"paymentdone","paymentnotdone")</f>
+        <v>paymentdone</v>
+      </c>
+      <c r="U3" t="str">
+        <f t="shared" ref="U3:U41" si="6">IF(K3&lt;15000,"low",IF(K3&lt;=30000,"medium",IF(K3&lt;=50000,"high","very high")))</f>
+        <v>high</v>
+      </c>
+      <c r="V3" t="str">
+        <f t="shared" ref="V3:V41" si="7">IF(AND(OR(E3="cardiology",E3="orthopedics"),K3&gt;30000),"management review","noreview")</f>
+        <v>management review</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -1605,8 +1697,44 @@
       <c r="M4">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:20">
+      <c r="N4" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O4" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P4" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q4" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R4" t="str">
+        <f t="shared" ref="R3:R41" si="8">IF(AND(L4="pending",K4&gt;30000),"follow-up","no action")</f>
+        <v>no action</v>
+      </c>
+      <c r="S4" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T4" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U4" t="str">
+        <f t="shared" si="6"/>
+        <v>low</v>
+      </c>
+      <c r="V4" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1646,8 +1774,44 @@
       <c r="M5">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:20">
+      <c r="N5" t="str">
+        <f t="shared" si="0"/>
+        <v>follow-up</v>
+      </c>
+      <c r="O5" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P5" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q5" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R5" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S5" t="str">
+        <f t="shared" si="4"/>
+        <v>priority dep</v>
+      </c>
+      <c r="T5" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentnotdone</v>
+      </c>
+      <c r="U5" t="str">
+        <f t="shared" si="6"/>
+        <v>medium</v>
+      </c>
+      <c r="V5" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -1687,8 +1851,44 @@
       <c r="M6">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:20">
+      <c r="N6" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O6" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P6" t="str">
+        <f t="shared" si="2"/>
+        <v>senior-citizen</v>
+      </c>
+      <c r="Q6" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R6" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S6" t="str">
+        <f t="shared" si="4"/>
+        <v>priority dep</v>
+      </c>
+      <c r="T6" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U6" t="str">
+        <f t="shared" si="6"/>
+        <v>medium</v>
+      </c>
+      <c r="V6" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -1728,8 +1928,44 @@
       <c r="M7">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:20">
+      <c r="N7" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O7" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P7" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q7" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R7" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S7" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T7" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U7" t="str">
+        <f t="shared" si="6"/>
+        <v>low</v>
+      </c>
+      <c r="V7" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -1769,8 +2005,44 @@
       <c r="M8">
         <v>9</v>
       </c>
-    </row>
-    <row r="9" spans="1:20">
+      <c r="N8" t="str">
+        <f t="shared" si="0"/>
+        <v>follow-up</v>
+      </c>
+      <c r="O8" t="str">
+        <f t="shared" si="1"/>
+        <v>high bill</v>
+      </c>
+      <c r="P8" t="str">
+        <f t="shared" si="2"/>
+        <v>senior-citizen</v>
+      </c>
+      <c r="Q8" t="str">
+        <f t="shared" si="3"/>
+        <v>High billing case</v>
+      </c>
+      <c r="R8" t="str">
+        <f t="shared" si="8"/>
+        <v>follow-up</v>
+      </c>
+      <c r="S8" t="str">
+        <f t="shared" si="4"/>
+        <v>priority dep</v>
+      </c>
+      <c r="T8" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentnotdone</v>
+      </c>
+      <c r="U8" t="str">
+        <f t="shared" si="6"/>
+        <v>very high</v>
+      </c>
+      <c r="V8" t="str">
+        <f t="shared" si="7"/>
+        <v>management review</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1810,8 +2082,44 @@
       <c r="M9">
         <v>2</v>
       </c>
-    </row>
-    <row r="10" spans="1:20">
+      <c r="N9" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O9" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P9" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q9" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R9" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S9" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T9" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U9" t="str">
+        <f t="shared" si="6"/>
+        <v>low</v>
+      </c>
+      <c r="V9" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1851,8 +2159,44 @@
       <c r="M10">
         <v>5</v>
       </c>
-    </row>
-    <row r="11" spans="1:20">
+      <c r="N10" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O10" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P10" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q10" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R10" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S10" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T10" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U10" t="str">
+        <f t="shared" si="6"/>
+        <v>medium</v>
+      </c>
+      <c r="V10" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -1892,8 +2236,44 @@
       <c r="M11">
         <v>2</v>
       </c>
-    </row>
-    <row r="12" spans="1:20">
+      <c r="N11" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O11" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P11" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q11" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R11" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S11" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T11" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U11" t="str">
+        <f t="shared" si="6"/>
+        <v>low</v>
+      </c>
+      <c r="V11" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -1933,8 +2313,44 @@
       <c r="M12">
         <v>4</v>
       </c>
-    </row>
-    <row r="13" spans="1:20">
+      <c r="N12" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O12" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P12" t="str">
+        <f t="shared" si="2"/>
+        <v>senior-citizen</v>
+      </c>
+      <c r="Q12" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R12" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S12" t="str">
+        <f t="shared" si="4"/>
+        <v>priority dep</v>
+      </c>
+      <c r="T12" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U12" t="str">
+        <f t="shared" si="6"/>
+        <v>medium</v>
+      </c>
+      <c r="V12" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -1974,8 +2390,44 @@
       <c r="M13">
         <v>7</v>
       </c>
-    </row>
-    <row r="14" spans="1:20">
+      <c r="N13" t="str">
+        <f t="shared" si="0"/>
+        <v>follow-up</v>
+      </c>
+      <c r="O13" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P13" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q13" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R13" t="str">
+        <f t="shared" si="8"/>
+        <v>follow-up</v>
+      </c>
+      <c r="S13" t="str">
+        <f t="shared" si="4"/>
+        <v>priority dep</v>
+      </c>
+      <c r="T13" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentnotdone</v>
+      </c>
+      <c r="U13" t="str">
+        <f t="shared" si="6"/>
+        <v>high</v>
+      </c>
+      <c r="V13" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -2015,8 +2467,44 @@
       <c r="M14">
         <v>3</v>
       </c>
-    </row>
-    <row r="15" spans="1:20">
+      <c r="N14" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O14" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P14" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q14" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R14" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S14" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T14" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U14" t="str">
+        <f t="shared" si="6"/>
+        <v>low</v>
+      </c>
+      <c r="V14" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -2056,8 +2544,44 @@
       <c r="M15">
         <v>4</v>
       </c>
-    </row>
-    <row r="16" spans="1:20">
+      <c r="N15" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O15" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P15" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q15" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R15" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S15" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T15" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U15" t="str">
+        <f t="shared" si="6"/>
+        <v>medium</v>
+      </c>
+      <c r="V15" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22">
       <c r="A16" t="s">
         <v>27</v>
       </c>
@@ -2097,8 +2621,44 @@
       <c r="M16">
         <v>10</v>
       </c>
-    </row>
-    <row r="17" spans="1:13">
+      <c r="N16" t="str">
+        <f t="shared" si="0"/>
+        <v>follow-up</v>
+      </c>
+      <c r="O16" t="str">
+        <f t="shared" si="1"/>
+        <v>high bill</v>
+      </c>
+      <c r="P16" t="str">
+        <f t="shared" si="2"/>
+        <v>senior-citizen</v>
+      </c>
+      <c r="Q16" t="str">
+        <f t="shared" si="3"/>
+        <v>High billing case</v>
+      </c>
+      <c r="R16" t="str">
+        <f t="shared" si="8"/>
+        <v>follow-up</v>
+      </c>
+      <c r="S16" t="str">
+        <f t="shared" si="4"/>
+        <v>priority dep</v>
+      </c>
+      <c r="T16" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentnotdone</v>
+      </c>
+      <c r="U16" t="str">
+        <f t="shared" si="6"/>
+        <v>very high</v>
+      </c>
+      <c r="V16" t="str">
+        <f t="shared" si="7"/>
+        <v>management review</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22">
       <c r="A17" t="s">
         <v>28</v>
       </c>
@@ -2138,8 +2698,44 @@
       <c r="M17">
         <v>3</v>
       </c>
-    </row>
-    <row r="18" spans="1:13">
+      <c r="N17" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O17" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P17" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q17" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R17" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S17" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T17" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U17" t="str">
+        <f t="shared" si="6"/>
+        <v>low</v>
+      </c>
+      <c r="V17" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22">
       <c r="A18" t="s">
         <v>29</v>
       </c>
@@ -2179,8 +2775,44 @@
       <c r="M18">
         <v>3</v>
       </c>
-    </row>
-    <row r="19" spans="1:13">
+      <c r="N18" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O18" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P18" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q18" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R18" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S18" t="str">
+        <f t="shared" si="4"/>
+        <v>priority dep</v>
+      </c>
+      <c r="T18" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U18" t="str">
+        <f t="shared" si="6"/>
+        <v>medium</v>
+      </c>
+      <c r="V18" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22">
       <c r="A19" t="s">
         <v>30</v>
       </c>
@@ -2220,8 +2852,44 @@
       <c r="M19">
         <v>8</v>
       </c>
-    </row>
-    <row r="20" spans="1:13">
+      <c r="N19" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O19" t="str">
+        <f t="shared" si="1"/>
+        <v>high bill</v>
+      </c>
+      <c r="P19" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q19" t="str">
+        <f t="shared" si="3"/>
+        <v>High billing case</v>
+      </c>
+      <c r="R19" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S19" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T19" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U19" t="str">
+        <f t="shared" si="6"/>
+        <v>high</v>
+      </c>
+      <c r="V19" t="str">
+        <f t="shared" si="7"/>
+        <v>management review</v>
+      </c>
+    </row>
+    <row r="20" spans="1:22">
       <c r="A20" t="s">
         <v>31</v>
       </c>
@@ -2261,8 +2929,44 @@
       <c r="M20">
         <v>2</v>
       </c>
-    </row>
-    <row r="21" spans="1:13">
+      <c r="N20" t="str">
+        <f t="shared" si="0"/>
+        <v>follow-up</v>
+      </c>
+      <c r="O20" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P20" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q20" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R20" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S20" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T20" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentnotdone</v>
+      </c>
+      <c r="U20" t="str">
+        <f t="shared" si="6"/>
+        <v>low</v>
+      </c>
+      <c r="V20" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22">
       <c r="A21" t="s">
         <v>32</v>
       </c>
@@ -2302,8 +3006,44 @@
       <c r="M21">
         <v>5</v>
       </c>
-    </row>
-    <row r="22" spans="1:13">
+      <c r="N21" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O21" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P21" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q21" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R21" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S21" t="str">
+        <f t="shared" si="4"/>
+        <v>priority dep</v>
+      </c>
+      <c r="T21" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U21" t="str">
+        <f t="shared" si="6"/>
+        <v>high</v>
+      </c>
+      <c r="V21" t="str">
+        <f t="shared" si="7"/>
+        <v>management review</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22">
       <c r="A22" t="s">
         <v>33</v>
       </c>
@@ -2343,8 +3083,44 @@
       <c r="M22">
         <v>3</v>
       </c>
-    </row>
-    <row r="23" spans="1:13">
+      <c r="N22" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O22" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P22" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q22" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R22" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S22" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T22" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U22" t="str">
+        <f t="shared" si="6"/>
+        <v>low</v>
+      </c>
+      <c r="V22" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22">
       <c r="A23" t="s">
         <v>34</v>
       </c>
@@ -2384,8 +3160,44 @@
       <c r="M23">
         <v>9</v>
       </c>
-    </row>
-    <row r="24" spans="1:13">
+      <c r="N23" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O23" t="str">
+        <f t="shared" si="1"/>
+        <v>high bill</v>
+      </c>
+      <c r="P23" t="str">
+        <f t="shared" si="2"/>
+        <v>senior-citizen</v>
+      </c>
+      <c r="Q23" t="str">
+        <f t="shared" si="3"/>
+        <v>High billing case</v>
+      </c>
+      <c r="R23" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S23" t="str">
+        <f t="shared" si="4"/>
+        <v>priority dep</v>
+      </c>
+      <c r="T23" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U23" t="str">
+        <f t="shared" si="6"/>
+        <v>high</v>
+      </c>
+      <c r="V23" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22">
       <c r="A24" t="s">
         <v>35</v>
       </c>
@@ -2425,8 +3237,44 @@
       <c r="M24">
         <v>3</v>
       </c>
-    </row>
-    <row r="25" spans="1:13">
+      <c r="N24" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O24" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P24" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q24" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R24" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S24" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T24" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U24" t="str">
+        <f t="shared" si="6"/>
+        <v>low</v>
+      </c>
+      <c r="V24" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22">
       <c r="A25" t="s">
         <v>36</v>
       </c>
@@ -2466,8 +3314,44 @@
       <c r="M25">
         <v>3</v>
       </c>
-    </row>
-    <row r="26" spans="1:13">
+      <c r="N25" t="str">
+        <f t="shared" si="0"/>
+        <v>follow-up</v>
+      </c>
+      <c r="O25" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P25" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q25" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R25" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S25" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T25" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentnotdone</v>
+      </c>
+      <c r="U25" t="str">
+        <f t="shared" si="6"/>
+        <v>medium</v>
+      </c>
+      <c r="V25" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22">
       <c r="A26" t="s">
         <v>37</v>
       </c>
@@ -2507,8 +3391,44 @@
       <c r="M26">
         <v>11</v>
       </c>
-    </row>
-    <row r="27" spans="1:13">
+      <c r="N26" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O26" t="str">
+        <f t="shared" si="1"/>
+        <v>high bill</v>
+      </c>
+      <c r="P26" t="str">
+        <f t="shared" si="2"/>
+        <v>senior-citizen</v>
+      </c>
+      <c r="Q26" t="str">
+        <f t="shared" si="3"/>
+        <v>High billing case</v>
+      </c>
+      <c r="R26" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S26" t="str">
+        <f t="shared" si="4"/>
+        <v>priority dep</v>
+      </c>
+      <c r="T26" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U26" t="str">
+        <f t="shared" si="6"/>
+        <v>very high</v>
+      </c>
+      <c r="V26" t="str">
+        <f t="shared" si="7"/>
+        <v>management review</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22">
       <c r="A27" t="s">
         <v>38</v>
       </c>
@@ -2548,8 +3468,44 @@
       <c r="M27">
         <v>2</v>
       </c>
-    </row>
-    <row r="28" spans="1:13">
+      <c r="N27" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O27" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P27" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q27" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R27" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S27" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T27" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U27" t="str">
+        <f t="shared" si="6"/>
+        <v>low</v>
+      </c>
+      <c r="V27" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="28" spans="1:22">
       <c r="A28" t="s">
         <v>39</v>
       </c>
@@ -2589,8 +3545,44 @@
       <c r="M28">
         <v>5</v>
       </c>
-    </row>
-    <row r="29" spans="1:13">
+      <c r="N28" t="str">
+        <f t="shared" si="0"/>
+        <v>follow-up</v>
+      </c>
+      <c r="O28" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P28" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q28" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R28" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S28" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T28" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentnotdone</v>
+      </c>
+      <c r="U28" t="str">
+        <f t="shared" si="6"/>
+        <v>medium</v>
+      </c>
+      <c r="V28" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="29" spans="1:22">
       <c r="A29" t="s">
         <v>40</v>
       </c>
@@ -2630,8 +3622,44 @@
       <c r="M29">
         <v>2</v>
       </c>
-    </row>
-    <row r="30" spans="1:13">
+      <c r="N29" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O29" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P29" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q29" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R29" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S29" t="str">
+        <f t="shared" si="4"/>
+        <v>priority dep</v>
+      </c>
+      <c r="T29" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U29" t="str">
+        <f t="shared" si="6"/>
+        <v>low</v>
+      </c>
+      <c r="V29" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22">
       <c r="A30" t="s">
         <v>41</v>
       </c>
@@ -2671,8 +3699,44 @@
       <c r="M30">
         <v>3</v>
       </c>
-    </row>
-    <row r="31" spans="1:13">
+      <c r="N30" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O30" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P30" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q30" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R30" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S30" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T30" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U30" t="str">
+        <f t="shared" si="6"/>
+        <v>low</v>
+      </c>
+      <c r="V30" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22">
       <c r="A31" t="s">
         <v>42</v>
       </c>
@@ -2712,8 +3776,44 @@
       <c r="M31">
         <v>4</v>
       </c>
-    </row>
-    <row r="32" spans="1:13">
+      <c r="N31" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O31" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P31" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q31" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R31" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S31" t="str">
+        <f t="shared" si="4"/>
+        <v>priority dep</v>
+      </c>
+      <c r="T31" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U31" t="str">
+        <f t="shared" si="6"/>
+        <v>medium</v>
+      </c>
+      <c r="V31" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="32" spans="1:22">
       <c r="A32" t="s">
         <v>43</v>
       </c>
@@ -2753,8 +3853,44 @@
       <c r="M32">
         <v>4</v>
       </c>
-    </row>
-    <row r="33" spans="1:13">
+      <c r="N32" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O32" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P32" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q32" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R32" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S32" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T32" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U32" t="str">
+        <f t="shared" si="6"/>
+        <v>low</v>
+      </c>
+      <c r="V32" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22">
       <c r="A33" t="s">
         <v>44</v>
       </c>
@@ -2794,8 +3930,44 @@
       <c r="M33">
         <v>7</v>
       </c>
-    </row>
-    <row r="34" spans="1:13">
+      <c r="N33" t="str">
+        <f t="shared" si="0"/>
+        <v>follow-up</v>
+      </c>
+      <c r="O33" t="str">
+        <f t="shared" si="1"/>
+        <v>high bill</v>
+      </c>
+      <c r="P33" t="str">
+        <f t="shared" si="2"/>
+        <v>senior-citizen</v>
+      </c>
+      <c r="Q33" t="str">
+        <f t="shared" si="3"/>
+        <v>High billing case</v>
+      </c>
+      <c r="R33" t="str">
+        <f t="shared" si="8"/>
+        <v>follow-up</v>
+      </c>
+      <c r="S33" t="str">
+        <f t="shared" si="4"/>
+        <v>priority dep</v>
+      </c>
+      <c r="T33" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentnotdone</v>
+      </c>
+      <c r="U33" t="str">
+        <f t="shared" si="6"/>
+        <v>high</v>
+      </c>
+      <c r="V33" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="34" spans="1:22">
       <c r="A34" t="s">
         <v>45</v>
       </c>
@@ -2835,8 +4007,44 @@
       <c r="M34">
         <v>9</v>
       </c>
-    </row>
-    <row r="35" spans="1:13">
+      <c r="N34" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O34" t="str">
+        <f t="shared" si="1"/>
+        <v>high bill</v>
+      </c>
+      <c r="P34" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q34" t="str">
+        <f t="shared" si="3"/>
+        <v>High billing case</v>
+      </c>
+      <c r="R34" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S34" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T34" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U34" t="str">
+        <f t="shared" si="6"/>
+        <v>high</v>
+      </c>
+      <c r="V34" t="str">
+        <f t="shared" si="7"/>
+        <v>management review</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22">
       <c r="A35" t="s">
         <v>46</v>
       </c>
@@ -2876,8 +4084,44 @@
       <c r="M35">
         <v>4</v>
       </c>
-    </row>
-    <row r="36" spans="1:13">
+      <c r="N35" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O35" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P35" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q35" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R35" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S35" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T35" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U35" t="str">
+        <f t="shared" si="6"/>
+        <v>medium</v>
+      </c>
+      <c r="V35" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22">
       <c r="A36" t="s">
         <v>47</v>
       </c>
@@ -2917,8 +4161,44 @@
       <c r="M36">
         <v>6</v>
       </c>
-    </row>
-    <row r="37" spans="1:13">
+      <c r="N36" t="str">
+        <f t="shared" si="0"/>
+        <v>follow-up</v>
+      </c>
+      <c r="O36" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P36" t="str">
+        <f t="shared" si="2"/>
+        <v>senior-citizen</v>
+      </c>
+      <c r="Q36" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R36" t="str">
+        <f t="shared" si="8"/>
+        <v>follow-up</v>
+      </c>
+      <c r="S36" t="str">
+        <f t="shared" si="4"/>
+        <v>priority dep</v>
+      </c>
+      <c r="T36" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentnotdone</v>
+      </c>
+      <c r="U36" t="str">
+        <f t="shared" si="6"/>
+        <v>high</v>
+      </c>
+      <c r="V36" t="str">
+        <f t="shared" si="7"/>
+        <v>management review</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22">
       <c r="A37" t="s">
         <v>48</v>
       </c>
@@ -2958,8 +4238,44 @@
       <c r="M37">
         <v>2</v>
       </c>
-    </row>
-    <row r="38" spans="1:13">
+      <c r="N37" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O37" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P37" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q37" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R37" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S37" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T37" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U37" t="str">
+        <f t="shared" si="6"/>
+        <v>low</v>
+      </c>
+      <c r="V37" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22">
       <c r="A38" t="s">
         <v>49</v>
       </c>
@@ -2999,8 +4315,44 @@
       <c r="M38">
         <v>4</v>
       </c>
-    </row>
-    <row r="39" spans="1:13">
+      <c r="N38" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O38" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P38" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q38" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R38" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S38" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T38" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U38" t="str">
+        <f t="shared" si="6"/>
+        <v>medium</v>
+      </c>
+      <c r="V38" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22">
       <c r="A39" t="s">
         <v>50</v>
       </c>
@@ -3040,8 +4392,44 @@
       <c r="M39">
         <v>2</v>
       </c>
-    </row>
-    <row r="40" spans="1:13">
+      <c r="N39" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O39" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P39" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q39" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R39" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S39" t="str">
+        <f t="shared" si="4"/>
+        <v>priority dep</v>
+      </c>
+      <c r="T39" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U39" t="str">
+        <f t="shared" si="6"/>
+        <v>low</v>
+      </c>
+      <c r="V39" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="40" spans="1:22">
       <c r="A40" t="s">
         <v>51</v>
       </c>
@@ -3081,8 +4469,44 @@
       <c r="M40">
         <v>4</v>
       </c>
-    </row>
-    <row r="41" spans="1:13">
+      <c r="N40" t="str">
+        <f t="shared" si="0"/>
+        <v>follow-up</v>
+      </c>
+      <c r="O40" t="str">
+        <f t="shared" si="1"/>
+        <v>normal bill</v>
+      </c>
+      <c r="P40" t="str">
+        <f t="shared" si="2"/>
+        <v>senior-citizen</v>
+      </c>
+      <c r="Q40" t="str">
+        <f t="shared" si="3"/>
+        <v>normal case</v>
+      </c>
+      <c r="R40" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S40" t="str">
+        <f t="shared" si="4"/>
+        <v>normaldep</v>
+      </c>
+      <c r="T40" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentnotdone</v>
+      </c>
+      <c r="U40" t="str">
+        <f t="shared" si="6"/>
+        <v>low</v>
+      </c>
+      <c r="V40" t="str">
+        <f t="shared" si="7"/>
+        <v>noreview</v>
+      </c>
+    </row>
+    <row r="41" spans="1:22">
       <c r="A41" t="s">
         <v>52</v>
       </c>
@@ -3122,14 +4546,50 @@
       <c r="M41">
         <v>10</v>
       </c>
-    </row>
-    <row r="43" spans="1:13">
+      <c r="N41" t="str">
+        <f t="shared" si="0"/>
+        <v>no action</v>
+      </c>
+      <c r="O41" t="str">
+        <f t="shared" si="1"/>
+        <v>high bill</v>
+      </c>
+      <c r="P41" t="str">
+        <f t="shared" si="2"/>
+        <v>non-senior</v>
+      </c>
+      <c r="Q41" t="str">
+        <f t="shared" si="3"/>
+        <v>High billing case</v>
+      </c>
+      <c r="R41" t="str">
+        <f t="shared" si="8"/>
+        <v>no action</v>
+      </c>
+      <c r="S41" t="str">
+        <f t="shared" si="4"/>
+        <v>priority dep</v>
+      </c>
+      <c r="T41" t="str">
+        <f t="shared" si="5"/>
+        <v>paymentdone</v>
+      </c>
+      <c r="U41" t="str">
+        <f t="shared" si="6"/>
+        <v>very high</v>
+      </c>
+      <c r="V41" t="str">
+        <f t="shared" si="7"/>
+        <v>management review</v>
+      </c>
+    </row>
+    <row r="43" spans="1:22">
       <c r="H43">
         <f>SUMIF(Department,"Opthomology",Bills)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:13">
+    <row r="47" spans="1:22">
       <c r="E47" t="s">
         <v>123</v>
       </c>
@@ -3138,7 +4598,7 @@
         <v>1019500</v>
       </c>
     </row>
-    <row r="48" spans="1:13">
+    <row r="48" spans="1:22">
       <c r="E48" t="s">
         <v>138</v>
       </c>
@@ -3301,9 +4761,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F0CC642-27D6-44E5-9163-DA270655D0F5}">
   <dimension ref="A1:C47"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="98.109375" customWidth="1"/>
+    <col min="1" max="1" width="98.08984375" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3516,11 +4976,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CC1AF7B-FEF6-4828-8271-552716DAF040}">
   <dimension ref="A1:D31"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="23.5546875" customWidth="1"/>
-    <col min="3" max="3" width="17.21875" customWidth="1"/>
-    <col min="4" max="4" width="21.109375" customWidth="1"/>
+    <col min="2" max="2" width="23.54296875" customWidth="1"/>
+    <col min="3" max="3" width="17.1796875" customWidth="1"/>
+    <col min="4" max="4" width="21.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -3915,7 +5375,7 @@
         <v>320000</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="28.8">
+    <row r="29" spans="1:4" ht="29">
       <c r="A29" s="3">
         <v>16</v>
       </c>

</xml_diff>